<commit_message>
Refresh NS5B RAS coverage annotations
</commit_message>
<xml_diff>
--- a/HCVData/Ref-selection/IncludedNS5BRefs_StatusInclude.xlsx
+++ b/HCVData/Ref-selection/IncludedNS5BRefs_StatusInclude.xlsx
@@ -618,13 +618,13 @@
         <v>777</v>
       </c>
       <c r="P2" s="1" t="n">
-        <v>431</v>
+        <v>777</v>
       </c>
       <c r="Q2" s="1" t="n">
-        <v>431</v>
+        <v>777</v>
       </c>
       <c r="R2" s="1" t="n">
-        <v>431</v>
+        <v>777</v>
       </c>
     </row>
     <row r="3">
@@ -686,13 +686,13 @@
         <v>443</v>
       </c>
       <c r="P3" s="1" t="n">
-        <v>0</v>
+        <v>443</v>
       </c>
       <c r="Q3" s="1" t="n">
-        <v>0</v>
+        <v>443</v>
       </c>
       <c r="R3" s="1" t="n">
-        <v>0</v>
+        <v>443</v>
       </c>
     </row>
     <row r="4">
@@ -754,13 +754,13 @@
         <v>71</v>
       </c>
       <c r="P4" s="1" t="n">
-        <v>141</v>
+        <v>71</v>
       </c>
       <c r="Q4" s="1" t="n">
-        <v>141</v>
+        <v>71</v>
       </c>
       <c r="R4" s="1" t="n">
-        <v>141</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5">
@@ -822,13 +822,13 @@
         <v>138</v>
       </c>
       <c r="P5" s="1" t="n">
-        <v>227</v>
+        <v>138</v>
       </c>
       <c r="Q5" s="1" t="n">
-        <v>227</v>
+        <v>138</v>
       </c>
       <c r="R5" s="1" t="n">
-        <v>227</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6">
@@ -890,13 +890,13 @@
         <v>123</v>
       </c>
       <c r="P6" s="1" t="n">
-        <v>211</v>
+        <v>123</v>
       </c>
       <c r="Q6" s="1" t="n">
-        <v>211</v>
+        <v>123</v>
       </c>
       <c r="R6" s="1" t="n">
-        <v>211</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
@@ -956,13 +956,13 @@
         <v>13</v>
       </c>
       <c r="P7" s="1" t="n">
-        <v>203</v>
+        <v>13</v>
       </c>
       <c r="Q7" s="1" t="n">
-        <v>203</v>
+        <v>13</v>
       </c>
       <c r="R7" s="1" t="n">
-        <v>203</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -1022,13 +1022,13 @@
         <v>18</v>
       </c>
       <c r="P8" s="1" t="n">
-        <v>200</v>
+        <v>18</v>
       </c>
       <c r="Q8" s="1" t="n">
-        <v>200</v>
+        <v>18</v>
       </c>
       <c r="R8" s="1" t="n">
-        <v>200</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -1090,13 +1090,13 @@
         <v>36</v>
       </c>
       <c r="P9" s="1" t="n">
-        <v>164</v>
+        <v>36</v>
       </c>
       <c r="Q9" s="1" t="n">
-        <v>164</v>
+        <v>36</v>
       </c>
       <c r="R9" s="1" t="n">
-        <v>164</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10">
@@ -1158,13 +1158,13 @@
         <v>94</v>
       </c>
       <c r="P10" s="1" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="Q10" s="1" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="R10" s="1" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11">
@@ -1226,13 +1226,13 @@
         <v>44</v>
       </c>
       <c r="P11" s="1" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="Q11" s="1" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="R11" s="1" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
@@ -1294,13 +1294,13 @@
         <v>514</v>
       </c>
       <c r="P12" s="1" t="n">
-        <v>0</v>
+        <v>511</v>
       </c>
       <c r="Q12" s="1" t="n">
-        <v>0</v>
+        <v>509</v>
       </c>
       <c r="R12" s="1" t="n">
-        <v>0</v>
+        <v>509</v>
       </c>
     </row>
     <row r="13">
@@ -1362,13 +1362,13 @@
         <v>8</v>
       </c>
       <c r="P13" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q13" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R13" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -1430,13 +1430,13 @@
         <v>12</v>
       </c>
       <c r="P14" s="1" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="Q14" s="1" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="R14" s="1" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -1498,13 +1498,13 @@
         <v>24</v>
       </c>
       <c r="P15" s="1" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="Q15" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R15" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -1566,13 +1566,13 @@
         <v>224</v>
       </c>
       <c r="P16" s="1" t="n">
-        <v>52</v>
+        <v>224</v>
       </c>
       <c r="Q16" s="1" t="n">
-        <v>52</v>
+        <v>224</v>
       </c>
       <c r="R16" s="1" t="n">
-        <v>52</v>
+        <v>224</v>
       </c>
     </row>
     <row r="17">
@@ -1636,13 +1636,13 @@
         <v>89</v>
       </c>
       <c r="P17" s="1" t="n">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="Q17" s="1" t="n">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="R17" s="1" t="n">
-        <v>8</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18">
@@ -1704,13 +1704,13 @@
         <v>71</v>
       </c>
       <c r="P18" s="1" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="Q18" s="1" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="R18" s="1" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19">
@@ -1766,13 +1766,13 @@
         <v>1</v>
       </c>
       <c r="P19" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R19" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1834,13 +1834,13 @@
         <v>182</v>
       </c>
       <c r="P20" s="1" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="Q20" s="1" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="R20" s="1" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
     </row>
     <row r="21">
@@ -1902,13 +1902,13 @@
         <v>26</v>
       </c>
       <c r="P21" s="1" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="Q21" s="1" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="R21" s="1" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22">
@@ -1974,13 +1974,13 @@
         <v>37</v>
       </c>
       <c r="P22" s="1" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="Q22" s="1" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="R22" s="1" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23">
@@ -2036,13 +2036,13 @@
         <v>1</v>
       </c>
       <c r="P23" s="1" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="Q23" s="1" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="R23" s="1" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -2104,13 +2104,13 @@
         <v>5</v>
       </c>
       <c r="P24" s="1" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="Q24" s="1" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="R24" s="1" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
@@ -2166,13 +2166,13 @@
         <v>324</v>
       </c>
       <c r="P25" s="1" t="n">
-        <v>0</v>
+        <v>321</v>
       </c>
       <c r="Q25" s="1" t="n">
-        <v>0</v>
+        <v>317</v>
       </c>
       <c r="R25" s="1" t="n">
-        <v>0</v>
+        <v>317</v>
       </c>
     </row>
     <row r="26">
@@ -2234,13 +2234,13 @@
         <v>101</v>
       </c>
       <c r="P26" s="1" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="Q26" s="1" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="R26" s="1" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27">
@@ -2302,13 +2302,13 @@
         <v>36</v>
       </c>
       <c r="P27" s="1" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="Q27" s="1" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="R27" s="1" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="28">
@@ -2370,13 +2370,13 @@
         <v>23</v>
       </c>
       <c r="P28" s="1" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="Q28" s="1" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="R28" s="1" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29">
@@ -2432,13 +2432,13 @@
         <v>1</v>
       </c>
       <c r="P29" s="1" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="Q29" s="1" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="R29" s="1" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -2500,13 +2500,13 @@
         <v>11</v>
       </c>
       <c r="P30" s="1" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="Q30" s="1" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="R30" s="1" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31">
@@ -2562,13 +2562,13 @@
         <v>1</v>
       </c>
       <c r="P31" s="1" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="Q31" s="1" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="R31" s="1" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -2622,13 +2622,13 @@
         <v>1</v>
       </c>
       <c r="P32" s="1" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="Q32" s="1" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R32" s="1" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -2690,13 +2690,13 @@
         <v>7</v>
       </c>
       <c r="P33" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q33" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="R33" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -2758,13 +2758,13 @@
         <v>35</v>
       </c>
       <c r="P34" s="1" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="Q34" s="1" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="R34" s="1" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35">
@@ -2826,13 +2826,13 @@
         <v>568</v>
       </c>
       <c r="P35" s="1" t="n">
-        <v>6</v>
+        <v>566</v>
       </c>
       <c r="Q35" s="1" t="n">
-        <v>6</v>
+        <v>560</v>
       </c>
       <c r="R35" s="1" t="n">
-        <v>6</v>
+        <v>559</v>
       </c>
     </row>
     <row r="36">
@@ -2886,13 +2886,13 @@
         <v>1</v>
       </c>
       <c r="P36" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q36" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R36" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -2946,13 +2946,13 @@
         <v>1</v>
       </c>
       <c r="P37" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q37" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R37" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -3014,13 +3014,13 @@
         <v>16</v>
       </c>
       <c r="P38" s="1" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="Q38" s="1" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="R38" s="1" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="39">
@@ -3076,13 +3076,13 @@
         <v>1</v>
       </c>
       <c r="P39" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q39" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R39" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -3144,13 +3144,13 @@
         <v>16</v>
       </c>
       <c r="P40" s="1" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="Q40" s="1" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="R40" s="1" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="41">
@@ -3212,13 +3212,13 @@
         <v>35</v>
       </c>
       <c r="P41" s="1" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="Q41" s="1" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="R41" s="1" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42">
@@ -3340,13 +3340,13 @@
         <v>57</v>
       </c>
       <c r="P43" s="1" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="Q43" s="1" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="R43" s="1" t="n">
-        <v>4</v>
+        <v>57</v>
       </c>
     </row>
     <row r="44">
@@ -3402,13 +3402,13 @@
         <v>1</v>
       </c>
       <c r="P44" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q44" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R44" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -3470,13 +3470,13 @@
         <v>6</v>
       </c>
       <c r="P45" s="1" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q45" s="1" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R45" s="1" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
@@ -3538,13 +3538,13 @@
         <v>62</v>
       </c>
       <c r="P46" s="1" t="n">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="Q46" s="1" t="n">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="R46" s="1" t="n">
-        <v>3</v>
+        <v>62</v>
       </c>
     </row>
     <row r="47">
@@ -3598,13 +3598,13 @@
         <v>1</v>
       </c>
       <c r="P47" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q47" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R47" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -3666,13 +3666,13 @@
         <v>7</v>
       </c>
       <c r="P48" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Q48" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="R48" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49">
@@ -3734,13 +3734,13 @@
         <v>20</v>
       </c>
       <c r="P49" s="1" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="Q49" s="1" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="R49" s="1" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50">
@@ -3798,13 +3798,13 @@
         <v>3</v>
       </c>
       <c r="P50" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q50" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R50" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -3866,13 +3866,13 @@
         <v>7</v>
       </c>
       <c r="P51" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q51" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="R51" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52">
@@ -4058,13 +4058,13 @@
         <v>1</v>
       </c>
       <c r="P54" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q54" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R54" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -4190,13 +4190,13 @@
         <v>43</v>
       </c>
       <c r="P56" s="1" t="n">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="Q56" s="1" t="n">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="R56" s="1" t="n">
-        <v>2</v>
+        <v>43</v>
       </c>
     </row>
     <row r="57">
@@ -4250,13 +4250,13 @@
         <v>1</v>
       </c>
       <c r="P57" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q57" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R57" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -4310,13 +4310,13 @@
         <v>1</v>
       </c>
       <c r="P58" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q58" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R58" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -4378,13 +4378,13 @@
         <v>78</v>
       </c>
       <c r="P59" s="1" t="n">
-        <v>2</v>
+        <v>78</v>
       </c>
       <c r="Q59" s="1" t="n">
-        <v>2</v>
+        <v>78</v>
       </c>
       <c r="R59" s="1" t="n">
-        <v>2</v>
+        <v>78</v>
       </c>
     </row>
     <row r="60">
@@ -4508,13 +4508,13 @@
         <v>14</v>
       </c>
       <c r="P61" s="1" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="Q61" s="1" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="R61" s="1" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="62">
@@ -4570,13 +4570,13 @@
         <v>1</v>
       </c>
       <c r="P62" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q62" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R62" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -4632,13 +4632,13 @@
         <v>1</v>
       </c>
       <c r="P63" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q63" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R63" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -4702,13 +4702,13 @@
         <v>10</v>
       </c>
       <c r="P64" s="1" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q64" s="1" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="R64" s="1" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65">
@@ -4762,13 +4762,13 @@
         <v>1</v>
       </c>
       <c r="P65" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q65" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R65" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -4830,13 +4830,13 @@
         <v>4</v>
       </c>
       <c r="P66" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q66" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R66" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67">
@@ -4962,13 +4962,13 @@
         <v>40</v>
       </c>
       <c r="P68" s="1" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="Q68" s="1" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="R68" s="1" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="69">
@@ -5026,13 +5026,13 @@
         <v>3</v>
       </c>
       <c r="P69" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q69" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R69" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -5156,13 +5156,13 @@
         <v>24</v>
       </c>
       <c r="P71" s="1" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="Q71" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R71" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="72">
@@ -5224,13 +5224,13 @@
         <v>14</v>
       </c>
       <c r="P72" s="1" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="Q72" s="1" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="R72" s="1" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="73">
@@ -5292,13 +5292,13 @@
         <v>6</v>
       </c>
       <c r="P73" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q73" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R73" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="74">
@@ -5474,13 +5474,13 @@
         <v>1</v>
       </c>
       <c r="P76" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q76" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R76" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -5542,13 +5542,13 @@
         <v>74</v>
       </c>
       <c r="P77" s="1" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="Q77" s="1" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="R77" s="1" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
     </row>
     <row r="78">
@@ -5610,13 +5610,13 @@
         <v>7</v>
       </c>
       <c r="P78" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q78" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R78" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79">
@@ -5678,13 +5678,13 @@
         <v>9</v>
       </c>
       <c r="P79" s="1" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="Q79" s="1" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="R79" s="1" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="80">
@@ -5746,13 +5746,13 @@
         <v>4</v>
       </c>
       <c r="P80" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q80" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R80" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81">
@@ -5808,13 +5808,13 @@
         <v>2</v>
       </c>
       <c r="P81" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q81" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R81" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
@@ -5876,13 +5876,13 @@
         <v>5</v>
       </c>
       <c r="P82" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q82" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R82" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="83">
@@ -5938,13 +5938,13 @@
         <v>3</v>
       </c>
       <c r="P83" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q83" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R83" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84">
@@ -6006,13 +6006,13 @@
         <v>14</v>
       </c>
       <c r="P84" s="1" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="Q84" s="1" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="R84" s="1" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="85">
@@ -6074,13 +6074,13 @@
         <v>11</v>
       </c>
       <c r="P85" s="1" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="Q85" s="1" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="R85" s="1" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="86">
@@ -6142,13 +6142,13 @@
         <v>31</v>
       </c>
       <c r="P86" s="1" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Q86" s="1" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="R86" s="1" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="87">
@@ -6210,13 +6210,13 @@
         <v>18</v>
       </c>
       <c r="P87" s="1" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="Q87" s="1" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="R87" s="1" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="88">
@@ -6278,13 +6278,13 @@
         <v>11</v>
       </c>
       <c r="P88" s="1" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="Q88" s="1" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="R88" s="1" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="89">
@@ -6346,13 +6346,13 @@
         <v>15</v>
       </c>
       <c r="P89" s="1" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="Q89" s="1" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="R89" s="1" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="90">
@@ -6414,13 +6414,13 @@
         <v>6</v>
       </c>
       <c r="P90" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q90" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R90" s="1" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="91">
@@ -6474,13 +6474,13 @@
         <v>1</v>
       </c>
       <c r="P91" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q91" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R91" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -6728,13 +6728,13 @@
         <v>13</v>
       </c>
       <c r="P95" s="1" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="Q95" s="1" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="R95" s="1" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="96">
@@ -6790,13 +6790,13 @@
         <v>1</v>
       </c>
       <c r="P96" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q96" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R96" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
@@ -6850,13 +6850,13 @@
         <v>1</v>
       </c>
       <c r="P97" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q97" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R97" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -6918,13 +6918,13 @@
         <v>14</v>
       </c>
       <c r="P98" s="1" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="Q98" s="1" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="R98" s="1" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="99">
@@ -6986,13 +6986,13 @@
         <v>10</v>
       </c>
       <c r="P99" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q99" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R99" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="100">
@@ -7054,13 +7054,13 @@
         <v>8</v>
       </c>
       <c r="P100" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q100" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R100" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="101">
@@ -7122,13 +7122,13 @@
         <v>10</v>
       </c>
       <c r="P101" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q101" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R101" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="102">
@@ -7188,13 +7188,13 @@
         <v>2</v>
       </c>
       <c r="P102" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q102" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R102" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103">
@@ -7248,13 +7248,13 @@
         <v>3</v>
       </c>
       <c r="P103" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q103" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R103" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="104">
@@ -7316,13 +7316,13 @@
         <v>5</v>
       </c>
       <c r="P104" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q104" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R104" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="105">
@@ -7382,13 +7382,13 @@
         <v>4</v>
       </c>
       <c r="P105" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q105" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R105" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106">
@@ -7450,13 +7450,13 @@
         <v>20</v>
       </c>
       <c r="P106" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q106" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R106" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="107">
@@ -7518,13 +7518,13 @@
         <v>31</v>
       </c>
       <c r="P107" s="1" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="Q107" s="1" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="R107" s="1" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
     </row>
     <row r="108">
@@ -7648,13 +7648,13 @@
         <v>3</v>
       </c>
       <c r="P109" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q109" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R109" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="110">
@@ -7718,13 +7718,13 @@
         <v>5</v>
       </c>
       <c r="P110" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q110" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R110" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="111">
@@ -7842,13 +7842,13 @@
         <v>3</v>
       </c>
       <c r="P112" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q112" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R112" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="113">
@@ -7906,13 +7906,13 @@
         <v>3</v>
       </c>
       <c r="P113" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q113" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R113" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="114">
@@ -7974,13 +7974,13 @@
         <v>77</v>
       </c>
       <c r="P114" s="1" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Q114" s="1" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="R114" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="115">
@@ -8160,13 +8160,13 @@
         <v>3</v>
       </c>
       <c r="P117" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q117" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R117" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="118">
@@ -8228,13 +8228,13 @@
         <v>9</v>
       </c>
       <c r="P118" s="1" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="Q118" s="1" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="R118" s="1" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="119">
@@ -8296,13 +8296,13 @@
         <v>26</v>
       </c>
       <c r="P119" s="1" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="Q119" s="1" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="R119" s="1" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="120">
@@ -8484,13 +8484,13 @@
         <v>2</v>
       </c>
       <c r="P122" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q122" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R122" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123">
@@ -8552,13 +8552,13 @@
         <v>120</v>
       </c>
       <c r="P123" s="1" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="Q123" s="1" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="R123" s="1" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="124">
@@ -8676,13 +8676,13 @@
         <v>2</v>
       </c>
       <c r="P125" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q125" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R125" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="126">
@@ -8804,13 +8804,13 @@
         <v>5</v>
       </c>
       <c r="P127" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q127" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R127" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="128">
@@ -8872,13 +8872,13 @@
         <v>6</v>
       </c>
       <c r="P128" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q128" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="R128" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="129">
@@ -8940,13 +8940,13 @@
         <v>45</v>
       </c>
       <c r="P129" s="1" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="Q129" s="1" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="R129" s="1" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
     </row>
     <row r="130">
@@ -9008,13 +9008,13 @@
         <v>20</v>
       </c>
       <c r="P130" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="Q130" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R130" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="131">
@@ -9074,13 +9074,13 @@
         <v>2</v>
       </c>
       <c r="P131" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q131" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R131" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="132">
@@ -9142,13 +9142,13 @@
         <v>4</v>
       </c>
       <c r="P132" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q132" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R132" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="133">
@@ -9204,13 +9204,13 @@
         <v>1</v>
       </c>
       <c r="P133" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q133" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R133" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -9270,13 +9270,13 @@
         <v>2</v>
       </c>
       <c r="P134" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q134" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R134" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="135">
@@ -9338,13 +9338,13 @@
         <v>8</v>
       </c>
       <c r="P135" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q135" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R135" s="1" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="136">
@@ -9406,13 +9406,13 @@
         <v>22</v>
       </c>
       <c r="P136" s="1" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="Q136" s="1" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="R136" s="1" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="137">
@@ -9472,13 +9472,13 @@
         <v>60</v>
       </c>
       <c r="P137" s="1" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="Q137" s="1" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="R137" s="1" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="138">
@@ -9540,13 +9540,13 @@
         <v>18</v>
       </c>
       <c r="P138" s="1" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="Q138" s="1" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="R138" s="1" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="139">
@@ -9600,13 +9600,13 @@
         <v>1</v>
       </c>
       <c r="P139" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q139" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R139" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140">
@@ -9664,13 +9664,13 @@
         <v>2</v>
       </c>
       <c r="P140" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q140" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R140" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="141">
@@ -9728,13 +9728,13 @@
         <v>1</v>
       </c>
       <c r="P141" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q141" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R141" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142">
@@ -9796,13 +9796,13 @@
         <v>11</v>
       </c>
       <c r="P142" s="1" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="Q142" s="1" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="R142" s="1" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="143">
@@ -9864,13 +9864,13 @@
         <v>7</v>
       </c>
       <c r="P143" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q143" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="R143" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="144">
@@ -9928,13 +9928,13 @@
         <v>2</v>
       </c>
       <c r="P144" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q144" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R144" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145">
@@ -10058,13 +10058,13 @@
         <v>1</v>
       </c>
       <c r="P146" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q146" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R146" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -10126,13 +10126,13 @@
         <v>6</v>
       </c>
       <c r="P147" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q147" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="R147" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="148">
@@ -10256,13 +10256,13 @@
         <v>22</v>
       </c>
       <c r="P149" s="1" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="Q149" s="1" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="R149" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="150">
@@ -10324,13 +10324,13 @@
         <v>60</v>
       </c>
       <c r="P150" s="1" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="Q150" s="1" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="R150" s="1" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
     </row>
     <row r="151">
@@ -10392,13 +10392,13 @@
         <v>25</v>
       </c>
       <c r="P151" s="1" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="Q151" s="1" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="R151" s="1" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="152">
@@ -10514,13 +10514,13 @@
         <v>3</v>
       </c>
       <c r="P153" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q153" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R153" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="154">
@@ -10582,13 +10582,13 @@
         <v>20</v>
       </c>
       <c r="P154" s="1" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="Q154" s="1" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="R154" s="1" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="155">
@@ -10712,13 +10712,13 @@
         <v>16</v>
       </c>
       <c r="P156" s="1" t="n">
-        <v>403</v>
+        <v>16</v>
       </c>
       <c r="Q156" s="1" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="R156" s="1" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="157">
@@ -10780,13 +10780,13 @@
         <v>8</v>
       </c>
       <c r="P157" s="1" t="n">
-        <v>321</v>
+        <v>8</v>
       </c>
       <c r="Q157" s="1" t="n">
-        <v>317</v>
+        <v>8</v>
       </c>
       <c r="R157" s="1" t="n">
-        <v>317</v>
+        <v>8</v>
       </c>
     </row>
     <row r="158">
@@ -10844,13 +10844,13 @@
         <v>5</v>
       </c>
       <c r="P158" s="1" t="n">
-        <v>265</v>
+        <v>5</v>
       </c>
       <c r="Q158" s="1" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R158" s="1" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="159">
@@ -10906,13 +10906,13 @@
         <v>2</v>
       </c>
       <c r="P159" s="1" t="n">
-        <v>224</v>
+        <v>2</v>
       </c>
       <c r="Q159" s="1" t="n">
-        <v>224</v>
+        <v>2</v>
       </c>
       <c r="R159" s="1" t="n">
-        <v>224</v>
+        <v>2</v>
       </c>
     </row>
     <row r="160">
@@ -10974,13 +10974,13 @@
         <v>9</v>
       </c>
       <c r="P160" s="1" t="n">
-        <v>182</v>
+        <v>9</v>
       </c>
       <c r="Q160" s="1" t="n">
-        <v>182</v>
+        <v>9</v>
       </c>
       <c r="R160" s="1" t="n">
-        <v>182</v>
+        <v>9</v>
       </c>
     </row>
     <row r="161">
@@ -11034,13 +11034,13 @@
         <v>1</v>
       </c>
       <c r="P161" s="1" t="n">
-        <v>138</v>
+        <v>1</v>
       </c>
       <c r="Q161" s="1" t="n">
-        <v>138</v>
+        <v>1</v>
       </c>
       <c r="R161" s="1" t="n">
-        <v>138</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162">
@@ -11102,13 +11102,13 @@
         <v>6</v>
       </c>
       <c r="P162" s="1" t="n">
-        <v>78</v>
+        <v>6</v>
       </c>
       <c r="Q162" s="1" t="n">
-        <v>78</v>
+        <v>6</v>
       </c>
       <c r="R162" s="1" t="n">
-        <v>78</v>
+        <v>6</v>
       </c>
     </row>
     <row r="163">
@@ -11164,13 +11164,13 @@
         <v>1</v>
       </c>
       <c r="P163" s="1" t="n">
-        <v>124</v>
+        <v>1</v>
       </c>
       <c r="Q163" s="1" t="n">
-        <v>124</v>
+        <v>1</v>
       </c>
       <c r="R163" s="1" t="n">
-        <v>124</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164">
@@ -11226,13 +11226,13 @@
         <v>1</v>
       </c>
       <c r="P164" s="1" t="n">
-        <v>120</v>
+        <v>1</v>
       </c>
       <c r="Q164" s="1" t="n">
-        <v>120</v>
+        <v>1</v>
       </c>
       <c r="R164" s="1" t="n">
-        <v>120</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165">
@@ -11286,13 +11286,13 @@
         <v>1</v>
       </c>
       <c r="P165" s="1" t="n">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="Q165" s="1" t="n">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="R165" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="166">
@@ -11348,13 +11348,13 @@
         <v>2</v>
       </c>
       <c r="P166" s="1" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="Q166" s="1" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="R166" s="1" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
@@ -11416,13 +11416,13 @@
         <v>12</v>
       </c>
       <c r="P167" s="1" t="n">
-        <v>95</v>
+        <v>12</v>
       </c>
       <c r="Q167" s="1" t="n">
-        <v>95</v>
+        <v>12</v>
       </c>
       <c r="R167" s="1" t="n">
-        <v>95</v>
+        <v>12</v>
       </c>
     </row>
     <row r="168">
@@ -11482,13 +11482,13 @@
         <v>1</v>
       </c>
       <c r="P168" s="1" t="n">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="Q168" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R168" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169">
@@ -11542,13 +11542,13 @@
         <v>1</v>
       </c>
       <c r="P169" s="1" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="Q169" s="1" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="R169" s="1" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170">
@@ -11610,13 +11610,13 @@
         <v>2</v>
       </c>
       <c r="P170" s="1" t="n">
-        <v>66</v>
+        <v>2</v>
       </c>
       <c r="Q170" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R170" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="171">
@@ -11676,13 +11676,13 @@
         <v>4</v>
       </c>
       <c r="P171" s="1" t="n">
-        <v>46</v>
+        <v>4</v>
       </c>
       <c r="Q171" s="1" t="n">
-        <v>46</v>
+        <v>4</v>
       </c>
       <c r="R171" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="172">
@@ -11738,13 +11738,13 @@
         <v>1</v>
       </c>
       <c r="P172" s="1" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="Q172" s="1" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="R172" s="1" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173">
@@ -11804,13 +11804,13 @@
         <v>1</v>
       </c>
       <c r="P173" s="1" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="Q173" s="1" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="R173" s="1" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174">
@@ -11868,13 +11868,13 @@
         <v>1</v>
       </c>
       <c r="P174" s="1" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="Q174" s="1" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="R174" s="1" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175">
@@ -11932,13 +11932,13 @@
         <v>2</v>
       </c>
       <c r="P175" s="1" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="Q175" s="1" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="R175" s="1" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="176">
@@ -11996,13 +11996,13 @@
         <v>4</v>
       </c>
       <c r="P176" s="1" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="Q176" s="1" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="R176" s="1" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
     </row>
     <row r="177">
@@ -12132,13 +12132,13 @@
         <v>73</v>
       </c>
       <c r="P178" s="1" t="n">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="Q178" s="1" t="n">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="R178" s="1" t="n">
-        <v>36</v>
+        <v>73</v>
       </c>
     </row>
     <row r="179">
@@ -12200,13 +12200,13 @@
         <v>50</v>
       </c>
       <c r="P179" s="1" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="Q179" s="1" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="R179" s="1" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="180">
@@ -12266,13 +12266,13 @@
         <v>4</v>
       </c>
       <c r="P180" s="1" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="Q180" s="1" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="R180" s="1" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
     </row>
     <row r="181">
@@ -12334,13 +12334,13 @@
         <v>1</v>
       </c>
       <c r="P181" s="1" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="Q181" s="1" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="R181" s="1" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -12394,13 +12394,13 @@
         <v>1</v>
       </c>
       <c r="P182" s="1" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="Q182" s="1" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="R182" s="1" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -12454,13 +12454,13 @@
         <v>1</v>
       </c>
       <c r="P183" s="1" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="Q183" s="1" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="R183" s="1" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184">
@@ -12514,13 +12514,13 @@
         <v>1</v>
       </c>
       <c r="P184" s="1" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="Q184" s="1" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="R184" s="1" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185">
@@ -12574,13 +12574,13 @@
         <v>1</v>
       </c>
       <c r="P185" s="1" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="Q185" s="1" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="R185" s="1" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="186">
@@ -12640,13 +12640,13 @@
         <v>2</v>
       </c>
       <c r="P186" s="1" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q186" s="1" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R186" s="1" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="187">
@@ -12700,13 +12700,13 @@
         <v>1</v>
       </c>
       <c r="P187" s="1" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="Q187" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R187" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188">
@@ -12762,13 +12762,13 @@
         <v>1</v>
       </c>
       <c r="P188" s="1" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="Q188" s="1" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="R188" s="1" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="189">
@@ -12824,13 +12824,13 @@
         <v>2</v>
       </c>
       <c r="P189" s="1" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="Q189" s="1" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="R189" s="1" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190">
@@ -12884,13 +12884,13 @@
         <v>1</v>
       </c>
       <c r="P190" s="1" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="Q190" s="1" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="R190" s="1" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="191">
@@ -12946,13 +12946,13 @@
         <v>1</v>
       </c>
       <c r="P191" s="1" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="Q191" s="1" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="R191" s="1" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -13006,13 +13006,13 @@
         <v>1</v>
       </c>
       <c r="P192" s="1" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="Q192" s="1" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="R192" s="1" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -13068,13 +13068,13 @@
         <v>1</v>
       </c>
       <c r="P193" s="1" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="Q193" s="1" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="R193" s="1" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194">
@@ -13130,13 +13130,13 @@
         <v>1</v>
       </c>
       <c r="P194" s="1" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="Q194" s="1" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="R194" s="1" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -13198,13 +13198,13 @@
         <v>15</v>
       </c>
       <c r="P195" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q195" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R195" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="196">
@@ -13268,13 +13268,13 @@
         <v>28</v>
       </c>
       <c r="P196" s="1" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="Q196" s="1" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="R196" s="1" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="197">
@@ -13336,13 +13336,13 @@
         <v>46</v>
       </c>
       <c r="P197" s="1" t="n">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="Q197" s="1" t="n">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="R197" s="1" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198">
@@ -13404,13 +13404,13 @@
         <v>100</v>
       </c>
       <c r="P198" s="1" t="n">
-        <v>11</v>
+        <v>97</v>
       </c>
       <c r="Q198" s="1" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="R198" s="1" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
     </row>
     <row r="199">
@@ -13472,13 +13472,13 @@
         <v>16</v>
       </c>
       <c r="P199" s="1" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="Q199" s="1" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="R199" s="1" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="200">
@@ -13540,13 +13540,13 @@
         <v>4</v>
       </c>
       <c r="P200" s="1" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="Q200" s="1" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="R200" s="1" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="201">
@@ -13608,13 +13608,13 @@
         <v>85</v>
       </c>
       <c r="P201" s="1" t="n">
-        <v>9</v>
+        <v>78</v>
       </c>
       <c r="Q201" s="1" t="n">
-        <v>9</v>
+        <v>78</v>
       </c>
       <c r="R201" s="1" t="n">
-        <v>9</v>
+        <v>78</v>
       </c>
     </row>
     <row r="202">
@@ -13678,13 +13678,13 @@
         <v>108</v>
       </c>
       <c r="P202" s="1" t="n">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="Q202" s="1" t="n">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="R202" s="1" t="n">
-        <v>6</v>
+        <v>107</v>
       </c>
     </row>
     <row r="203">
@@ -13746,13 +13746,13 @@
         <v>26</v>
       </c>
       <c r="P203" s="1" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="Q203" s="1" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="R203" s="1" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="204">
@@ -13808,13 +13808,13 @@
         <v>1</v>
       </c>
       <c r="P204" s="1" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q204" s="1" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R204" s="1" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205">
@@ -13870,13 +13870,13 @@
         <v>4</v>
       </c>
       <c r="P205" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q205" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R205" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="206">
@@ -13938,13 +13938,13 @@
         <v>33</v>
       </c>
       <c r="P206" s="1" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="Q206" s="1" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="R206" s="1" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
     </row>
     <row r="207">
@@ -14006,13 +14006,13 @@
         <v>330</v>
       </c>
       <c r="P207" s="1" t="n">
-        <v>1</v>
+        <v>279</v>
       </c>
       <c r="Q207" s="1" t="n">
-        <v>1</v>
+        <v>265</v>
       </c>
       <c r="R207" s="1" t="n">
-        <v>1</v>
+        <v>265</v>
       </c>
     </row>
     <row r="208">
@@ -14074,13 +14074,13 @@
         <v>31</v>
       </c>
       <c r="P208" s="1" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="Q208" s="1" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="R208" s="1" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
     </row>
     <row r="209">
@@ -14142,13 +14142,13 @@
         <v>12</v>
       </c>
       <c r="P209" s="1" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="Q209" s="1" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="R209" s="1" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="210">
@@ -14210,13 +14210,13 @@
         <v>71</v>
       </c>
       <c r="P210" s="1" t="n">
-        <v>1</v>
+        <v>66</v>
       </c>
       <c r="Q210" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R210" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="211">
@@ -14278,13 +14278,13 @@
         <v>84</v>
       </c>
       <c r="P211" s="1" t="n">
-        <v>3</v>
+        <v>84</v>
       </c>
       <c r="Q211" s="1" t="n">
-        <v>3</v>
+        <v>84</v>
       </c>
       <c r="R211" s="1" t="n">
-        <v>3</v>
+        <v>84</v>
       </c>
     </row>
     <row r="212">
@@ -14340,13 +14340,13 @@
         <v>3</v>
       </c>
       <c r="P212" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q212" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R212" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="213">
@@ -14404,13 +14404,13 @@
         <v>21</v>
       </c>
       <c r="P213" s="1" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Q213" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R213" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="214">
@@ -14474,13 +14474,13 @@
         <v>41</v>
       </c>
       <c r="P214" s="1" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="Q214" s="1" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="R214" s="1" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
     </row>
     <row r="215">
@@ -14542,13 +14542,13 @@
         <v>108</v>
       </c>
       <c r="P215" s="1" t="n">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="Q215" s="1" t="n">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="R215" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="216">
@@ -14612,13 +14612,13 @@
         <v>1556</v>
       </c>
       <c r="P216" s="1" t="n">
-        <v>2</v>
+        <v>1556</v>
       </c>
       <c r="Q216" s="1" t="n">
-        <v>2</v>
+        <v>1556</v>
       </c>
       <c r="R216" s="1" t="n">
-        <v>2</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="217">
@@ -14682,13 +14682,13 @@
         <v>511</v>
       </c>
       <c r="P217" s="1" t="n">
-        <v>2</v>
+        <v>511</v>
       </c>
       <c r="Q217" s="1" t="n">
-        <v>2</v>
+        <v>511</v>
       </c>
       <c r="R217" s="1" t="n">
-        <v>2</v>
+        <v>511</v>
       </c>
     </row>
     <row r="218">
@@ -14742,13 +14742,13 @@
         <v>1</v>
       </c>
       <c r="P218" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q218" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R218" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219">
@@ -14806,13 +14806,13 @@
         <v>3</v>
       </c>
       <c r="P219" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q219" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R219" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220">
@@ -14874,13 +14874,13 @@
         <v>11</v>
       </c>
       <c r="P220" s="1" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="Q220" s="1" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="R220" s="1" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="221">
@@ -14942,13 +14942,13 @@
         <v>124</v>
       </c>
       <c r="P221" s="1" t="n">
-        <v>1</v>
+        <v>124</v>
       </c>
       <c r="Q221" s="1" t="n">
-        <v>1</v>
+        <v>124</v>
       </c>
       <c r="R221" s="1" t="n">
-        <v>1</v>
+        <v>124</v>
       </c>
     </row>
     <row r="222">
@@ -15012,13 +15012,13 @@
         <v>87</v>
       </c>
       <c r="P222" s="1" t="n">
-        <v>1</v>
+        <v>87</v>
       </c>
       <c r="Q222" s="1" t="n">
-        <v>1</v>
+        <v>87</v>
       </c>
       <c r="R222" s="1" t="n">
-        <v>1</v>
+        <v>87</v>
       </c>
     </row>
     <row r="223">
@@ -15080,13 +15080,13 @@
         <v>12</v>
       </c>
       <c r="P223" s="1" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="Q223" s="1" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="R223" s="1" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="224">
@@ -15148,13 +15148,13 @@
         <v>35</v>
       </c>
       <c r="P224" s="1" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="Q224" s="1" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="R224" s="1" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
     </row>
     <row r="225">
@@ -15216,13 +15216,13 @@
         <v>3</v>
       </c>
       <c r="P225" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q225" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R225" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="226">
@@ -15284,13 +15284,13 @@
         <v>107</v>
       </c>
       <c r="P226" s="1" t="n">
-        <v>1</v>
+        <v>107</v>
       </c>
       <c r="Q226" s="1" t="n">
-        <v>1</v>
+        <v>107</v>
       </c>
       <c r="R226" s="1" t="n">
-        <v>1</v>
+        <v>107</v>
       </c>
     </row>
     <row r="227">
@@ -15354,13 +15354,13 @@
         <v>281</v>
       </c>
       <c r="P227" s="1" t="n">
-        <v>1</v>
+        <v>265</v>
       </c>
       <c r="Q227" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R227" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="228">
@@ -15418,13 +15418,13 @@
         <v>2</v>
       </c>
       <c r="P228" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q228" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R228" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="229">
@@ -15486,13 +15486,13 @@
         <v>14</v>
       </c>
       <c r="P229" s="1" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="Q229" s="1" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="R229" s="1" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="230">
@@ -15554,13 +15554,13 @@
         <v>10</v>
       </c>
       <c r="P230" s="1" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Q230" s="1" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="R230" s="1" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="231">
@@ -15622,13 +15622,13 @@
         <v>8</v>
       </c>
       <c r="P231" s="1" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="Q231" s="1" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="R231" s="1" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="232">
@@ -15690,13 +15690,13 @@
         <v>132</v>
       </c>
       <c r="P232" s="1" t="n">
-        <v>1</v>
+        <v>132</v>
       </c>
       <c r="Q232" s="1" t="n">
-        <v>1</v>
+        <v>132</v>
       </c>
       <c r="R232" s="1" t="n">
-        <v>1</v>
+        <v>131</v>
       </c>
     </row>
     <row r="233">
@@ -15758,13 +15758,13 @@
         <v>14</v>
       </c>
       <c r="P233" s="1" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="Q233" s="1" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="R233" s="1" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="234">
@@ -15826,13 +15826,13 @@
         <v>433</v>
       </c>
       <c r="P234" s="1" t="n">
-        <v>1556</v>
+        <v>403</v>
       </c>
       <c r="Q234" s="1" t="n">
-        <v>1556</v>
+        <v>0</v>
       </c>
       <c r="R234" s="1" t="n">
-        <v>1556</v>
+        <v>0</v>
       </c>
     </row>
     <row r="235">
@@ -15894,13 +15894,13 @@
         <v>24</v>
       </c>
       <c r="P235" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Q235" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R235" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="236">
@@ -15962,7 +15962,7 @@
         <v>95</v>
       </c>
       <c r="P236" s="1" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="Q236" s="1" t="n">
         <v>0</v>
@@ -16032,13 +16032,13 @@
         <v>80</v>
       </c>
       <c r="P237" s="1" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="Q237" s="1" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="R237" s="1" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="238">
@@ -16100,13 +16100,13 @@
         <v>95</v>
       </c>
       <c r="P238" s="1" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="Q238" s="1" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="R238" s="1" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
     </row>
     <row r="239">
@@ -16168,7 +16168,7 @@
         <v>19</v>
       </c>
       <c r="P239" s="1" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="Q239" s="1" t="n">
         <v>0</v>
@@ -16236,7 +16236,7 @@
         <v>9</v>
       </c>
       <c r="P240" s="1" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="Q240" s="1" t="n">
         <v>0</v>
@@ -16304,13 +16304,13 @@
         <v>113</v>
       </c>
       <c r="P241" s="1" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="Q241" s="1" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="R241" s="1" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
     </row>
     <row r="242">
@@ -16372,13 +16372,13 @@
         <v>1</v>
       </c>
       <c r="P242" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q242" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R242" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="243">
@@ -16440,13 +16440,13 @@
         <v>10</v>
       </c>
       <c r="P243" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q243" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R243" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="244">
@@ -16504,13 +16504,13 @@
         <v>164</v>
       </c>
       <c r="P244" s="1" t="n">
-        <v>23</v>
+        <v>163</v>
       </c>
       <c r="Q244" s="1" t="n">
-        <v>20</v>
+        <v>163</v>
       </c>
       <c r="R244" s="1" t="n">
-        <v>18</v>
+        <v>109</v>
       </c>
     </row>
     <row r="245">
@@ -16570,7 +16570,7 @@
         <v>613</v>
       </c>
       <c r="P245" s="1" t="n">
-        <v>0</v>
+        <v>574</v>
       </c>
       <c r="Q245" s="1" t="n">
         <v>0</v>
@@ -16634,13 +16634,13 @@
         <v>1</v>
       </c>
       <c r="P246" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q246" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R246" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="247">
@@ -16702,13 +16702,13 @@
         <v>67</v>
       </c>
       <c r="P247" s="1" t="n">
-        <v>3</v>
+        <v>67</v>
       </c>
       <c r="Q247" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R247" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248">

</xml_diff>